<commit_message>
chore : upload du dossier de code du projet
</commit_message>
<xml_diff>
--- a/RoadMap Projet/Planning_et_deroule_2025_2026 (1).xlsx
+++ b/RoadMap Projet/Planning_et_deroule_2025_2026 (1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keuni\Desktop\ESIGELEC\Cours\Programmer_en_java\PDL ESIGELEC\RoadMap Projet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50D563B3-0AB5-4A18-9FB5-49745E8AB6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0997432A-D301-42B7-93E3-240884A6707C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="16440" tabRatio="758" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="4" r:id="rId1"/>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="65">
   <si>
     <t>Cours</t>
   </si>
@@ -833,6 +833,12 @@
       <alignment textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -842,15 +848,15 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -860,28 +866,22 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1188,132 +1188,132 @@
     <row r="1" spans="1:92" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="4"/>
-      <c r="C1" s="59" t="s">
+      <c r="C1" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="59" t="s">
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="59" t="s">
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="64"/>
+      <c r="M1" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="63" t="s">
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="64"/>
+      <c r="R1" s="65" t="s">
         <v>21</v>
       </c>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="64"/>
-      <c r="V1" s="69"/>
-      <c r="W1" s="59" t="s">
+      <c r="S1" s="66"/>
+      <c r="T1" s="66"/>
+      <c r="U1" s="66"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="62" t="s">
         <v>8</v>
       </c>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="62"/>
-      <c r="AB1" s="59" t="s">
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="64"/>
+      <c r="AB1" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="60"/>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="62"/>
-      <c r="AG1" s="59" t="s">
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="63"/>
+      <c r="AE1" s="63"/>
+      <c r="AF1" s="64"/>
+      <c r="AG1" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="AH1" s="60"/>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="60"/>
-      <c r="AK1" s="62"/>
-      <c r="AL1" s="59" t="s">
+      <c r="AH1" s="63"/>
+      <c r="AI1" s="63"/>
+      <c r="AJ1" s="63"/>
+      <c r="AK1" s="64"/>
+      <c r="AL1" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="AM1" s="60"/>
-      <c r="AN1" s="60"/>
-      <c r="AO1" s="60"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="59" t="s">
+      <c r="AM1" s="63"/>
+      <c r="AN1" s="63"/>
+      <c r="AO1" s="63"/>
+      <c r="AP1" s="64"/>
+      <c r="AQ1" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="AR1" s="60"/>
-      <c r="AS1" s="60"/>
-      <c r="AT1" s="60"/>
-      <c r="AU1" s="62"/>
-      <c r="AV1" s="59" t="s">
+      <c r="AR1" s="63"/>
+      <c r="AS1" s="63"/>
+      <c r="AT1" s="63"/>
+      <c r="AU1" s="64"/>
+      <c r="AV1" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="AW1" s="60"/>
-      <c r="AX1" s="60"/>
-      <c r="AY1" s="60"/>
-      <c r="AZ1" s="61"/>
-      <c r="BA1" s="59" t="s">
+      <c r="AW1" s="63"/>
+      <c r="AX1" s="63"/>
+      <c r="AY1" s="63"/>
+      <c r="AZ1" s="72"/>
+      <c r="BA1" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="62"/>
-      <c r="BF1" s="63" t="s">
+      <c r="BB1" s="63"/>
+      <c r="BC1" s="63"/>
+      <c r="BD1" s="63"/>
+      <c r="BE1" s="64"/>
+      <c r="BF1" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="BG1" s="64"/>
-      <c r="BH1" s="64"/>
-      <c r="BI1" s="64"/>
-      <c r="BJ1" s="65"/>
-      <c r="BK1" s="63" t="s">
+      <c r="BG1" s="66"/>
+      <c r="BH1" s="66"/>
+      <c r="BI1" s="66"/>
+      <c r="BJ1" s="71"/>
+      <c r="BK1" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="BL1" s="64"/>
-      <c r="BM1" s="64"/>
-      <c r="BN1" s="64"/>
-      <c r="BO1" s="65"/>
-      <c r="BP1" s="70" t="s">
+      <c r="BL1" s="66"/>
+      <c r="BM1" s="66"/>
+      <c r="BN1" s="66"/>
+      <c r="BO1" s="71"/>
+      <c r="BP1" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="BQ1" s="71"/>
-      <c r="BR1" s="71"/>
-      <c r="BS1" s="71"/>
-      <c r="BT1" s="72"/>
-      <c r="BU1" s="59" t="s">
+      <c r="BQ1" s="69"/>
+      <c r="BR1" s="69"/>
+      <c r="BS1" s="69"/>
+      <c r="BT1" s="70"/>
+      <c r="BU1" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="BV1" s="60"/>
-      <c r="BW1" s="60"/>
-      <c r="BX1" s="60"/>
-      <c r="BY1" s="62"/>
-      <c r="BZ1" s="56" t="s">
+      <c r="BV1" s="63"/>
+      <c r="BW1" s="63"/>
+      <c r="BX1" s="63"/>
+      <c r="BY1" s="64"/>
+      <c r="BZ1" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="CA1" s="57"/>
-      <c r="CB1" s="57"/>
-      <c r="CC1" s="57"/>
-      <c r="CD1" s="58"/>
-      <c r="CE1" s="56" t="s">
+      <c r="CA1" s="59"/>
+      <c r="CB1" s="59"/>
+      <c r="CC1" s="59"/>
+      <c r="CD1" s="60"/>
+      <c r="CE1" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="CF1" s="57"/>
-      <c r="CG1" s="57"/>
-      <c r="CH1" s="57"/>
-      <c r="CI1" s="58"/>
-      <c r="CJ1" s="56" t="s">
+      <c r="CF1" s="59"/>
+      <c r="CG1" s="59"/>
+      <c r="CH1" s="59"/>
+      <c r="CI1" s="60"/>
+      <c r="CJ1" s="58" t="s">
         <v>43</v>
       </c>
-      <c r="CK1" s="57"/>
-      <c r="CL1" s="57"/>
-      <c r="CM1" s="57"/>
-      <c r="CN1" s="58"/>
+      <c r="CK1" s="59"/>
+      <c r="CL1" s="59"/>
+      <c r="CM1" s="59"/>
+      <c r="CN1" s="60"/>
     </row>
     <row r="2" spans="1:92" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2107,6 +2107,18 @@
       <c r="AH9" t="s">
         <v>64</v>
       </c>
+      <c r="AI9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>63</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="10" spans="1:92" ht="255" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C10" s="28" t="s">
@@ -2297,102 +2309,102 @@
       </c>
     </row>
     <row r="11" spans="1:92" x14ac:dyDescent="0.25">
-      <c r="C11" s="68" t="s">
+      <c r="C11" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="D11" s="68"/>
-      <c r="E11" s="68"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
-      <c r="I11" s="68"/>
-      <c r="J11" s="68"/>
-      <c r="K11" s="68"/>
-      <c r="L11" s="68"/>
-      <c r="M11" s="68"/>
-      <c r="N11" s="68"/>
-      <c r="O11" s="68"/>
-      <c r="P11" s="68"/>
-      <c r="Q11" s="68"/>
-      <c r="R11" s="68"/>
-      <c r="S11" s="68"/>
-      <c r="T11" s="68"/>
-      <c r="U11" s="68"/>
-      <c r="V11" s="68"/>
-      <c r="W11" s="68"/>
-      <c r="X11" s="68"/>
-      <c r="Y11" s="68"/>
-      <c r="Z11" s="68"/>
-      <c r="AA11" s="68"/>
-      <c r="AB11" s="68"/>
-      <c r="AC11" s="68"/>
-      <c r="AD11" s="68"/>
-      <c r="AE11" s="68"/>
-      <c r="AF11" s="68"/>
-      <c r="AG11" s="67" t="s">
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="61"/>
+      <c r="L11" s="61"/>
+      <c r="M11" s="61"/>
+      <c r="N11" s="61"/>
+      <c r="O11" s="61"/>
+      <c r="P11" s="61"/>
+      <c r="Q11" s="61"/>
+      <c r="R11" s="61"/>
+      <c r="S11" s="61"/>
+      <c r="T11" s="61"/>
+      <c r="U11" s="61"/>
+      <c r="V11" s="61"/>
+      <c r="W11" s="61"/>
+      <c r="X11" s="61"/>
+      <c r="Y11" s="61"/>
+      <c r="Z11" s="61"/>
+      <c r="AA11" s="61"/>
+      <c r="AB11" s="61"/>
+      <c r="AC11" s="61"/>
+      <c r="AD11" s="61"/>
+      <c r="AE11" s="61"/>
+      <c r="AF11" s="61"/>
+      <c r="AG11" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="AH11" s="67"/>
-      <c r="AI11" s="67"/>
-      <c r="AJ11" s="67"/>
-      <c r="AK11" s="67"/>
-      <c r="AL11" s="67"/>
-      <c r="AM11" s="67"/>
-      <c r="AN11" s="67"/>
-      <c r="AO11" s="67"/>
-      <c r="AP11" s="67"/>
-      <c r="AQ11" s="67"/>
-      <c r="AR11" s="67"/>
-      <c r="AS11" s="67"/>
-      <c r="AT11" s="67"/>
-      <c r="AU11" s="67"/>
-      <c r="AV11" s="67"/>
-      <c r="AW11" s="67"/>
-      <c r="AX11" s="67"/>
-      <c r="AY11" s="67"/>
-      <c r="AZ11" s="67"/>
-      <c r="BA11" s="67"/>
-      <c r="BB11" s="67"/>
-      <c r="BC11" s="67"/>
-      <c r="BD11" s="67"/>
-      <c r="BE11" s="67"/>
-      <c r="BF11" s="67"/>
-      <c r="BG11" s="67"/>
-      <c r="BH11" s="67"/>
-      <c r="BI11" s="67"/>
-      <c r="BJ11" s="67"/>
-      <c r="BK11" s="67"/>
-      <c r="BL11" s="67"/>
-      <c r="BM11" s="67"/>
-      <c r="BN11" s="67"/>
-      <c r="BO11" s="67"/>
-      <c r="BP11" s="67"/>
-      <c r="BQ11" s="67"/>
-      <c r="BR11" s="67"/>
-      <c r="BS11" s="67"/>
-      <c r="BT11" s="67"/>
-      <c r="BU11" s="67"/>
-      <c r="BV11" s="67"/>
-      <c r="BW11" s="67"/>
-      <c r="BX11" s="67"/>
-      <c r="BY11" s="67"/>
-      <c r="BZ11" s="67"/>
-      <c r="CA11" s="67"/>
-      <c r="CB11" s="67"/>
-      <c r="CC11" s="67"/>
-      <c r="CD11" s="67"/>
-      <c r="CE11" s="66" t="s">
+      <c r="AH11" s="57"/>
+      <c r="AI11" s="57"/>
+      <c r="AJ11" s="57"/>
+      <c r="AK11" s="57"/>
+      <c r="AL11" s="57"/>
+      <c r="AM11" s="57"/>
+      <c r="AN11" s="57"/>
+      <c r="AO11" s="57"/>
+      <c r="AP11" s="57"/>
+      <c r="AQ11" s="57"/>
+      <c r="AR11" s="57"/>
+      <c r="AS11" s="57"/>
+      <c r="AT11" s="57"/>
+      <c r="AU11" s="57"/>
+      <c r="AV11" s="57"/>
+      <c r="AW11" s="57"/>
+      <c r="AX11" s="57"/>
+      <c r="AY11" s="57"/>
+      <c r="AZ11" s="57"/>
+      <c r="BA11" s="57"/>
+      <c r="BB11" s="57"/>
+      <c r="BC11" s="57"/>
+      <c r="BD11" s="57"/>
+      <c r="BE11" s="57"/>
+      <c r="BF11" s="57"/>
+      <c r="BG11" s="57"/>
+      <c r="BH11" s="57"/>
+      <c r="BI11" s="57"/>
+      <c r="BJ11" s="57"/>
+      <c r="BK11" s="57"/>
+      <c r="BL11" s="57"/>
+      <c r="BM11" s="57"/>
+      <c r="BN11" s="57"/>
+      <c r="BO11" s="57"/>
+      <c r="BP11" s="57"/>
+      <c r="BQ11" s="57"/>
+      <c r="BR11" s="57"/>
+      <c r="BS11" s="57"/>
+      <c r="BT11" s="57"/>
+      <c r="BU11" s="57"/>
+      <c r="BV11" s="57"/>
+      <c r="BW11" s="57"/>
+      <c r="BX11" s="57"/>
+      <c r="BY11" s="57"/>
+      <c r="BZ11" s="57"/>
+      <c r="CA11" s="57"/>
+      <c r="CB11" s="57"/>
+      <c r="CC11" s="57"/>
+      <c r="CD11" s="57"/>
+      <c r="CE11" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="CF11" s="66"/>
-      <c r="CG11" s="66"/>
-      <c r="CH11" s="66"/>
-      <c r="CI11" s="66"/>
-      <c r="CJ11" s="66"/>
-      <c r="CK11" s="66"/>
-      <c r="CL11" s="66"/>
-      <c r="CM11" s="66"/>
-      <c r="CN11" s="66"/>
+      <c r="CF11" s="56"/>
+      <c r="CG11" s="56"/>
+      <c r="CH11" s="56"/>
+      <c r="CI11" s="56"/>
+      <c r="CJ11" s="56"/>
+      <c r="CK11" s="56"/>
+      <c r="CL11" s="56"/>
+      <c r="CM11" s="56"/>
+      <c r="CN11" s="56"/>
     </row>
     <row r="13" spans="1:92" x14ac:dyDescent="0.25">
       <c r="C13" s="15"/>
@@ -2429,6 +2441,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="CE1:CI1"/>
+    <mergeCell ref="AV1:AZ1"/>
+    <mergeCell ref="BA1:BE1"/>
+    <mergeCell ref="BF1:BJ1"/>
+    <mergeCell ref="BZ1:CD1"/>
     <mergeCell ref="CE11:CN11"/>
     <mergeCell ref="AG11:CD11"/>
     <mergeCell ref="CJ1:CN1"/>
@@ -2445,11 +2462,6 @@
     <mergeCell ref="BP1:BT1"/>
     <mergeCell ref="BU1:BY1"/>
     <mergeCell ref="BK1:BO1"/>
-    <mergeCell ref="CE1:CI1"/>
-    <mergeCell ref="AV1:AZ1"/>
-    <mergeCell ref="BA1:BE1"/>
-    <mergeCell ref="BF1:BJ1"/>
-    <mergeCell ref="BZ1:CD1"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>